<commit_message>
Rename Clubs to Teams across the site; add Find & replace to admin
- All site wording now says Teams (Media Team, Preferred team, ...);
  page links and ids are unchanged (clubs.html still works)
- Admin > Tools > Find & replace: change a word everywhere at once,
  keeping capitals; never touches links, images or ids
- {team} works in the success message alongside {club}
- Sheet template and Apps Script use team names/headings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps-script/CSS-Recruitment.xlsx
+++ b/apps-script/CSS-Recruitment.xlsx
@@ -578,12 +578,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Preferred club</t>
+          <t>Preferred team</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Secondary club</t>
+          <t>Secondary team</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -12634,7 +12634,7 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -12651,7 +12651,7 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Media Club</t>
+          <t>Media Team</t>
         </is>
       </c>
       <c r="B7" s="11">
@@ -12666,7 +12666,7 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Graphics Club</t>
+          <t>Graphics Team</t>
         </is>
       </c>
       <c r="B8" s="13">
@@ -12681,7 +12681,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Operations Club</t>
+          <t>Operations Team</t>
         </is>
       </c>
       <c r="B9" s="11">
@@ -12696,7 +12696,7 @@
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Events Club</t>
+          <t>Events Team</t>
         </is>
       </c>
       <c r="B10" s="13">
@@ -12711,7 +12711,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Decor Club</t>
+          <t>Decor Team</t>
         </is>
       </c>
       <c r="B11" s="11">
@@ -12969,7 +12969,7 @@
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
         <is>
-          <t>Club, department and semester lists come from the website's current content. If you rename a club or department in the admin, update it here too.</t>
+          <t>Team, department and semester lists come from the website's current content. If you rename a team or department in the admin, update it here too.</t>
         </is>
       </c>
     </row>
@@ -13152,14 +13152,14 @@
     <row r="23">
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Preferred club:  Graphics Club</t>
+          <t>Preferred team:  Graphics Team</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="20" t="inlineStr">
         <is>
-          <t>Secondary club:  Media Club</t>
+          <t>Secondary team:  Media Team</t>
         </is>
       </c>
     </row>

</xml_diff>